<commit_message>
feat(dofa): add verified 6-band conformal prediction reports, per-class coverage & summary metrics
Co-authored-by: Claude <claude@anthropic.com>
</commit_message>
<xml_diff>
--- a/Classification/dofa/results/uncertainty_results/conformal_reports_all_models.xlsx
+++ b/Classification/dofa/results/uncertainty_results/conformal_reports_all_models.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="104">
   <si>
     <t>model_name</t>
   </si>
@@ -151,22 +151,19 @@
     <t>timestamp_utc</t>
   </si>
   <si>
-    <t>/content/drive/My Drive/Classification/data/data.csv</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/data/ref.csv</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/dofa/models</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/dofa/results/uncertainty_results</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/dofa/results</t>
-  </si>
-  <si>
-    <t>2026-08-18T06:37:06.535452+00:00</t>
+    <t>/kaggle/input/datasets/daneshselwal/dias-6-bands-data/k001.csv</t>
+  </si>
+  <si>
+    <t>/kaggle/input/datasets/daneshselwal/dias-6-bands-data/k002.csv</t>
+  </si>
+  <si>
+    <t>/kaggle/input</t>
+  </si>
+  <si>
+    <t>/kaggle/working/Classification/dofa/results/uncertainty_results</t>
+  </si>
+  <si>
+    <t>2026-10-11T12:56:29.587768+00:00</t>
   </si>
   <si>
     <t>SplitConformal - DOFA_Spectral</t>
@@ -2934,28 +2931,28 @@
         <v>0.95</v>
       </c>
       <c r="D2">
-        <v>0.9568445475638051</v>
+        <v>0.9517401392111369</v>
       </c>
       <c r="E2">
-        <v>0.9568445475638051</v>
+        <v>0.9517401392111369</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>0.9568445475638051</v>
+        <v>0.9517401392111369</v>
       </c>
       <c r="H2">
-        <v>0.0431554524361949</v>
+        <v>0.04825986078886311</v>
       </c>
       <c r="I2">
-        <v>1.488178547999723</v>
+        <v>1.918234962000042</v>
       </c>
       <c r="J2">
         <v>0.05</v>
       </c>
       <c r="M2">
-        <v>0.9585245644320887</v>
+        <v>0.9578829616138655</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2984,7 +2981,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>1.487060923999707</v>
+        <v>1.781241131999991</v>
       </c>
       <c r="J3">
         <v>0.05</v>
@@ -3004,28 +3001,28 @@
         <v>0.95</v>
       </c>
       <c r="D4">
-        <v>0.9651972157772621</v>
+        <v>0.9573085846867749</v>
       </c>
       <c r="E4">
-        <v>0.965661252900232</v>
+        <v>0.9577726218097448</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>0.965661252900232</v>
+        <v>0.9577726218097448</v>
       </c>
       <c r="H4">
-        <v>0.03433874709976798</v>
+        <v>0.04222737819025522</v>
       </c>
       <c r="I4">
-        <v>1.469506139000259</v>
+        <v>1.589364872999965</v>
       </c>
       <c r="J4">
         <v>0.05</v>
       </c>
       <c r="M4">
-        <v>0.9656427257933603</v>
+        <v>0.9632547675729706</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -3039,22 +3036,22 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="E5">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="H5">
-        <v>0.04640371229698376</v>
+        <v>0.04872389791183294</v>
       </c>
       <c r="I5">
-        <v>8.468704089000312</v>
+        <v>6.860590443999968</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -3063,7 +3060,7 @@
         <v>4</v>
       </c>
       <c r="M5">
-        <v>0.9610824551190823</v>
+        <v>0.9577474497896404</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3092,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>2.090471408999747</v>
+        <v>2.146093229999963</v>
       </c>
       <c r="J6">
         <v>0.05</v>
@@ -3115,22 +3112,22 @@
         <v>0.95</v>
       </c>
       <c r="D7">
-        <v>0.9633410672853828</v>
+        <v>0.9577726218097448</v>
       </c>
       <c r="E7">
-        <v>0.9633410672853828</v>
+        <v>0.9582366589327146</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>0.9633410672853828</v>
+        <v>0.9582366589327146</v>
       </c>
       <c r="H7">
-        <v>0.03665893271461717</v>
+        <v>0.04176334106728538</v>
       </c>
       <c r="I7">
-        <v>6.484488911999961</v>
+        <v>5.404915652999989</v>
       </c>
       <c r="J7">
         <v>0.05</v>
@@ -3139,7 +3136,7 @@
         <v>4</v>
       </c>
       <c r="M7">
-        <v>0.9641101485684878</v>
+        <v>0.9635694308832286</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -3153,7 +3150,7 @@
         <v>0.95</v>
       </c>
       <c r="D8">
-        <v>0.9948955916473318</v>
+        <v>0.9944315545243619</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -3168,7 +3165,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>0.3806276049999724</v>
+        <v>0.4154801280000129</v>
       </c>
       <c r="J8">
         <v>0.05</v>
@@ -3177,7 +3174,7 @@
         <v>0.01</v>
       </c>
       <c r="M8">
-        <v>0.9925132328872037</v>
+        <v>0.9932433269064765</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3206,7 +3203,7 @@
         <v>0</v>
       </c>
       <c r="I9">
-        <v>0.3882359640001596</v>
+        <v>0.390346610999984</v>
       </c>
       <c r="J9">
         <v>0.05</v>
@@ -3229,7 +3226,7 @@
         <v>0.95</v>
       </c>
       <c r="D10">
-        <v>0.9962877030162413</v>
+        <v>0.9944315545243619</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -3244,7 +3241,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>0.3957724679999046</v>
+        <v>0.3811832259999619</v>
       </c>
       <c r="J10">
         <v>0.05</v>
@@ -3253,7 +3250,7 @@
         <v>0.01</v>
       </c>
       <c r="M10">
-        <v>0.9963725361616106</v>
+        <v>0.9928109972774349</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3267,28 +3264,28 @@
         <v>0.95</v>
       </c>
       <c r="D11">
-        <v>0.962877030162413</v>
+        <v>0.9573085846867749</v>
       </c>
       <c r="E11">
-        <v>0.962877030162413</v>
+        <v>0.9573085846867749</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11">
-        <v>0.962877030162413</v>
+        <v>0.9573085846867749</v>
       </c>
       <c r="H11">
-        <v>0.03712296983758701</v>
+        <v>0.04269141531322506</v>
       </c>
       <c r="I11">
-        <v>1.585017308999795</v>
+        <v>1.526185338999994</v>
       </c>
       <c r="J11">
         <v>0.05</v>
       </c>
       <c r="M11">
-        <v>0.9644779724609794</v>
+        <v>0.9654833336158465</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -3317,7 +3314,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>1.50854602399977</v>
+        <v>1.561271374</v>
       </c>
       <c r="J12">
         <v>0.05</v>
@@ -3337,28 +3334,28 @@
         <v>0.95</v>
       </c>
       <c r="D13">
-        <v>0.9675174013921114</v>
+        <v>0.9596287703016241</v>
       </c>
       <c r="E13">
-        <v>0.9679814385150812</v>
+        <v>0.960092807424594</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13">
-        <v>0.9679814385150812</v>
+        <v>0.960092807424594</v>
       </c>
       <c r="H13">
-        <v>0.03201856148491879</v>
+        <v>0.03990719257540603</v>
       </c>
       <c r="I13">
-        <v>1.990267985999708</v>
+        <v>1.54946296899999</v>
       </c>
       <c r="J13">
         <v>0.05</v>
       </c>
       <c r="M13">
-        <v>0.9701578041677665</v>
+        <v>0.964437369711878</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -3372,28 +3369,28 @@
         <v>0.95</v>
       </c>
       <c r="D14">
-        <v>0.9526682134570765</v>
+        <v>0.9498839907192576</v>
       </c>
       <c r="E14">
-        <v>0.9526682134570765</v>
+        <v>0.9498839907192576</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14">
-        <v>0.9526682134570765</v>
+        <v>0.9498839907192576</v>
       </c>
       <c r="H14">
-        <v>0.04733178654292344</v>
+        <v>0.05011600928074246</v>
       </c>
       <c r="I14">
-        <v>1.542094702000213</v>
+        <v>1.537332433000017</v>
       </c>
       <c r="J14">
         <v>0.05</v>
       </c>
       <c r="M14">
-        <v>0.9546024182297265</v>
+        <v>0.954647598587596</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -3422,7 +3419,7 @@
         <v>0</v>
       </c>
       <c r="I15">
-        <v>1.501472937000017</v>
+        <v>1.644036248999953</v>
       </c>
       <c r="J15">
         <v>0.05</v>
@@ -3442,28 +3439,28 @@
         <v>0.95</v>
       </c>
       <c r="D16">
-        <v>0.9568445475638051</v>
+        <v>0.9651972157772621</v>
       </c>
       <c r="E16">
-        <v>0.9568445475638051</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16">
-        <v>0.9568445475638051</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="H16">
-        <v>0.0431554524361949</v>
+        <v>0.03387470997679815</v>
       </c>
       <c r="I16">
-        <v>1.526485220000268</v>
+        <v>1.610437100000013</v>
       </c>
       <c r="J16">
         <v>0.05</v>
       </c>
       <c r="M16">
-        <v>0.9546740538134185</v>
+        <v>0.9602859023151588</v>
       </c>
     </row>
   </sheetData>
@@ -3478,15 +3475,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3541,44 +3538,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9675174013921114</v>
+        <v>0.9596287703016241</v>
       </c>
       <c r="E5">
-        <v>0.9679814385150812</v>
+        <v>0.960092807424594</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9679814385150812</v>
+        <v>0.960092807424594</v>
       </c>
       <c r="H5">
-        <v>0.03201856148491879</v>
+        <v>0.03990719257540603</v>
       </c>
       <c r="I5">
-        <v>1.990267985999708</v>
+        <v>1.54946296899999</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9701578041677665</v>
+        <v>0.964437369711878</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3586,7 +3583,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9638949671772429</v>
+        <v>0.949671772428884</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -3597,7 +3594,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9647577092511013</v>
+        <v>0.9669603524229075</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -3608,7 +3605,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9776536312849162</v>
+        <v>0.9720670391061452</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -3619,7 +3616,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9487179487179487</v>
+        <v>0.9358974358974359</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -3630,7 +3627,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>0.9903846153846154</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -3660,18 +3657,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -3679,10 +3676,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>34556</v>
+        <v>34500</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -3690,10 +3687,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>13814</v>
+        <v>13911</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -3701,10 +3698,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>15163</v>
+        <v>14355</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -3712,10 +3709,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>4263</v>
+        <v>3976</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -3723,13 +3720,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>3649</v>
+        <v>3652</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -3737,10 +3734,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>3359</v>
+        <v>4497</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -3748,10 +3745,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>2055</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -3759,26 +3756,26 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>24451</v>
+        <v>24273</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -3786,7 +3783,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.03699135784066721</v>
+        <v>0.03709699152069912</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -3797,7 +3794,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.04023779438175035</v>
+        <v>0.04105959648254087</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -3808,7 +3805,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.06328886747360229</v>
+        <v>0.04452757114297035</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -3819,7 +3816,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.04921856874059993</v>
+        <v>0.04464513419328209</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -3830,7 +3827,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.087204730549578</v>
+        <v>0.1235085195041559</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -3841,7 +3838,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.03965676309979804</v>
+        <v>0.05949343174777211</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -3852,7 +3849,7 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.06081736012957795</v>
+        <v>0.0557932543723958</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -3860,12 +3857,12 @@
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -3881,15 +3878,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3944,22 +3941,22 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9633410672853828</v>
+        <v>0.9577726218097448</v>
       </c>
       <c r="E5">
-        <v>0.9633410672853828</v>
+        <v>0.9582366589327146</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9633410672853828</v>
+        <v>0.9582366589327146</v>
       </c>
       <c r="H5">
-        <v>0.03665893271461717</v>
+        <v>0.04176334106728538</v>
       </c>
       <c r="I5">
-        <v>6.484488911999961</v>
+        <v>5.404915652999989</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -3968,23 +3965,23 @@
         <v>4</v>
       </c>
       <c r="M5">
-        <v>0.9641101485684878</v>
+        <v>0.9635694308832286</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3992,7 +3989,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9595185995623632</v>
+        <v>0.9463894967177243</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -4003,7 +4000,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9757709251101322</v>
+        <v>0.9669603524229075</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -4014,7 +4011,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9581005586592178</v>
+        <v>0.9692737430167597</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -4025,7 +4022,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9487179487179487</v>
+        <v>0.9358974358974359</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -4047,7 +4044,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9603960396039604</v>
+        <v>0.9801980198019802</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -4066,15 +4063,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -4117,7 +4114,7 @@
         <v>2</v>
       </c>
       <c r="J25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -4138,15 +4135,15 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -4154,7 +4151,7 @@
         <v>0</v>
       </c>
       <c r="B32">
-        <v>0.04339605516682721</v>
+        <v>0.04080493776715921</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -4162,7 +4159,7 @@
         <v>1</v>
       </c>
       <c r="B33">
-        <v>0.06081736012957795</v>
+        <v>0.0557932543723958</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -4170,7 +4167,7 @@
         <v>2</v>
       </c>
       <c r="B34">
-        <v>0.03687418628397643</v>
+        <v>0.03703275936966077</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -4178,20 +4175,20 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>0.03674598561303999</v>
+        <v>0.05435002715128745</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -4199,7 +4196,7 @@
         <v>0</v>
       </c>
       <c r="B40">
-        <v>0.9638802889576883</v>
+        <v>0.9638429752066116</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -4207,7 +4204,7 @@
         <v>1</v>
       </c>
       <c r="B41">
-        <v>0.9558823529411765</v>
+        <v>0.9701492537313433</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -4215,7 +4212,7 @@
         <v>2</v>
       </c>
       <c r="B42">
-        <v>0.962671905697446</v>
+        <v>0.9499509322865555</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -4223,20 +4220,20 @@
         <v>3</v>
       </c>
       <c r="B43">
-        <v>0.97</v>
+        <v>0.9801980198019802</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -4244,7 +4241,7 @@
         <v>0</v>
       </c>
       <c r="B48">
-        <v>0.9595185995623632</v>
+        <v>0.9453551912568307</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -4252,10 +4249,10 @@
         <v>1</v>
       </c>
       <c r="B49">
-        <v>0.977924944812362</v>
+        <v>0.977728285077951</v>
       </c>
       <c r="J49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -4263,7 +4260,7 @@
         <v>2</v>
       </c>
       <c r="B50">
-        <v>0.9527777777777777</v>
+        <v>0.9586776859504132</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -4271,7 +4268,7 @@
         <v>3</v>
       </c>
       <c r="B51">
-        <v>0.9487179487179487</v>
+        <v>0.9358974358974359</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -4287,7 +4284,7 @@
         <v>5</v>
       </c>
       <c r="B53">
-        <v>0.97</v>
+        <v>0.9801980198019802</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -4295,12 +4292,12 @@
         <v>6</v>
       </c>
       <c r="B54">
-        <v>0.9558823529411765</v>
+        <v>0.9701492537313433</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -4316,15 +4313,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4379,7 +4376,7 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9962877030162413</v>
+        <v>0.9944315545243619</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4394,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.3957724679999046</v>
+        <v>0.3811832259999619</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -4403,23 +4400,23 @@
         <v>0.01</v>
       </c>
       <c r="M5">
-        <v>0.9963725361616106</v>
+        <v>0.9928109972774349</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4438,7 +4435,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9911894273127754</v>
+        <v>0.9845814977973568</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -4449,7 +4446,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.994413407821229</v>
+        <v>0.9972067039106145</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -4460,7 +4457,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>0.9935897435897436</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -4493,7 +4490,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>0.9852941176470589</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -4501,18 +4498,18 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -4539,15 +4536,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4602,44 +4599,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9526682134570765</v>
+        <v>0.9498839907192576</v>
       </c>
       <c r="E5">
-        <v>0.9526682134570765</v>
+        <v>0.9498839907192576</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9526682134570765</v>
+        <v>0.9498839907192576</v>
       </c>
       <c r="H5">
-        <v>0.04733178654292344</v>
+        <v>0.05011600928074246</v>
       </c>
       <c r="I5">
-        <v>1.542094702000213</v>
+        <v>1.537332433000017</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9546024182297265</v>
+        <v>0.954647598587596</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4647,7 +4644,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9540481400437637</v>
+        <v>0.9529540481400438</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -4658,7 +4655,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9581497797356828</v>
+        <v>0.9273127753303965</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -4669,7 +4666,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9357541899441341</v>
+        <v>0.9581005586592178</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -4702,7 +4699,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9603960396039604</v>
+        <v>0.9702970297029703</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -4721,18 +4718,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -4740,10 +4737,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>34012</v>
+        <v>32865</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -4751,10 +4748,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>13165</v>
+        <v>13114</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -4762,10 +4759,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>13833</v>
+        <v>14978</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -4773,10 +4770,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>4258</v>
+        <v>4724</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -4784,13 +4781,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>3588</v>
+        <v>3368</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -4798,10 +4795,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>3235</v>
+        <v>3708</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -4809,10 +4806,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>1757</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -4820,35 +4817,35 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>27462</v>
+        <v>26963</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33">
-        <v>0.02959583517864617</v>
+        <v>0.03075113394702211</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -4864,15 +4861,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4927,44 +4924,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9568445475638051</v>
+        <v>0.9517401392111369</v>
       </c>
       <c r="E5">
-        <v>0.9568445475638051</v>
+        <v>0.9517401392111369</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9568445475638051</v>
+        <v>0.9517401392111369</v>
       </c>
       <c r="H5">
-        <v>0.0431554524361949</v>
+        <v>0.04825986078886311</v>
       </c>
       <c r="I5">
-        <v>1.488178547999723</v>
+        <v>1.918234962000042</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9585245644320887</v>
+        <v>0.9578829616138655</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4972,7 +4969,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9617067833698031</v>
+        <v>0.9540481400437637</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -4983,7 +4980,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9581497797356828</v>
+        <v>0.9405286343612335</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -4994,7 +4991,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9357541899441341</v>
+        <v>0.946927374301676</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -5005,7 +5002,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9615384615384616</v>
+        <v>0.9423076923076923</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -5016,7 +5013,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9615384615384616</v>
+        <v>0.9903846153846154</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -5046,18 +5043,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -5065,10 +5062,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>34456</v>
+        <v>33062</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -5076,10 +5073,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>13292</v>
+        <v>14110</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -5087,10 +5084,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>13837</v>
+        <v>13869</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -5098,10 +5095,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>4653</v>
+        <v>4670</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -5109,13 +5106,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>2970</v>
+        <v>3355</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -5123,10 +5120,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>3056</v>
+        <v>3348</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -5134,10 +5131,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>2320</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -5145,23 +5142,23 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>26726</v>
+        <v>26494</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -5169,7 +5166,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.02964517529469313</v>
+        <v>0.03078984717777389</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -5177,7 +5174,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.03023690300569126</v>
+        <v>0.0373079471750638</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -5185,7 +5182,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.02960675457756701</v>
+        <v>0.02707039426447488</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -5193,7 +5190,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.03302371344323407</v>
+        <v>0.0303705070607776</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -5201,7 +5198,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.02184981637932415</v>
+        <v>0.03009650968692079</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -5209,7 +5206,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.02701234344195236</v>
+        <v>0.02699720721266174</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -5217,17 +5214,17 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.1040660244560911</v>
+        <v>0.3320036111752476</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -5243,15 +5240,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5306,44 +5303,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.962877030162413</v>
+        <v>0.9573085846867749</v>
       </c>
       <c r="E5">
-        <v>0.962877030162413</v>
+        <v>0.9573085846867749</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.962877030162413</v>
+        <v>0.9573085846867749</v>
       </c>
       <c r="H5">
-        <v>0.03712296983758701</v>
+        <v>0.04269141531322506</v>
       </c>
       <c r="I5">
-        <v>1.585017308999795</v>
+        <v>1.526185338999994</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9644779724609794</v>
+        <v>0.9654833336158465</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -5351,7 +5348,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9660831509846827</v>
+        <v>0.9573304157549234</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -5362,7 +5359,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9647577092511013</v>
+        <v>0.9405286343612335</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -5373,7 +5370,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.946927374301676</v>
+        <v>0.9581005586592178</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -5395,7 +5392,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9711538461538461</v>
+        <v>1</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -5425,18 +5422,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -5444,10 +5441,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>34820</v>
+        <v>33278</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -5455,10 +5452,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>13432</v>
+        <v>14137</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -5466,10 +5463,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>14157</v>
+        <v>14869</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -5477,10 +5474,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>4670</v>
+        <v>5051</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -5488,13 +5485,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>3126</v>
+        <v>3488</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -5502,10 +5499,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>3950</v>
+        <v>3755</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -5513,10 +5510,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>2320</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -5524,26 +5521,26 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>24835</v>
+        <v>24330</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -5551,7 +5548,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.0296914152383152</v>
+        <v>0.03083860916014058</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -5562,7 +5559,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.0310858949254802</v>
+        <v>0.03756839395633738</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -5573,7 +5570,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.03048189391538991</v>
+        <v>0.0301658797852522</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -5584,7 +5581,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.03322517156101179</v>
+        <v>0.03400261402329297</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -5595,7 +5592,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.02269835665573816</v>
+        <v>0.0377494659292511</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -5606,7 +5603,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.04481606674520699</v>
+        <v>0.03137481979403089</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -5617,7 +5614,7 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.1040660244560911</v>
+        <v>0.3320036111752476</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -5625,12 +5622,12 @@
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -5646,15 +5643,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5709,22 +5706,22 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="E5">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="H5">
-        <v>0.04640371229698376</v>
+        <v>0.04872389791183294</v>
       </c>
       <c r="I5">
-        <v>8.468704089000312</v>
+        <v>6.860590443999968</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -5733,23 +5730,23 @@
         <v>4</v>
       </c>
       <c r="M5">
-        <v>0.9610824551190823</v>
+        <v>0.9577474497896404</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -5757,7 +5754,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9507658643326039</v>
+        <v>0.9551422319474836</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -5768,7 +5765,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9581497797356828</v>
+        <v>0.9273127753303965</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -5779,7 +5776,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9357541899441341</v>
+        <v>0.9581005586592178</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -5790,7 +5787,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9615384615384616</v>
+        <v>0.9423076923076923</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -5831,15 +5828,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -5882,7 +5879,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -5903,15 +5900,15 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -5919,7 +5916,7 @@
         <v>0</v>
       </c>
       <c r="B32">
-        <v>0.02957745344955165</v>
+        <v>0.03079497762998606</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -5927,7 +5924,7 @@
         <v>1</v>
       </c>
       <c r="B33">
-        <v>0.1040660244560911</v>
+        <v>0.3320036111752476</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -5935,7 +5932,7 @@
         <v>2</v>
       </c>
       <c r="B34">
-        <v>0.03302371344323407</v>
+        <v>0.0303705070607776</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -5943,20 +5940,20 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>0.02701234344195236</v>
+        <v>0.02699720721266174</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -5964,7 +5961,7 @@
         <v>0</v>
       </c>
       <c r="B40">
-        <v>0.9524330235101148</v>
+        <v>0.9523809523809523</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -5972,7 +5969,7 @@
         <v>1</v>
       </c>
       <c r="B41">
-        <v>1</v>
+        <v>0.9850746268656716</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -5980,7 +5977,7 @@
         <v>2</v>
       </c>
       <c r="B42">
-        <v>0.9554140127388535</v>
+        <v>0.91875</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -5988,20 +5985,20 @@
         <v>3</v>
       </c>
       <c r="B43">
-        <v>0.941747572815534</v>
+        <v>0.9603960396039604</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -6009,7 +6006,7 @@
         <v>0</v>
       </c>
       <c r="B48">
-        <v>0.9497267759562842</v>
+        <v>0.9561883899233297</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -6017,10 +6014,10 @@
         <v>1</v>
       </c>
       <c r="B49">
-        <v>0.9623893805309734</v>
+        <v>0.9376391982182628</v>
       </c>
       <c r="J49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -6028,7 +6025,7 @@
         <v>2</v>
       </c>
       <c r="B50">
-        <v>0.9357541899441341</v>
+        <v>0.9527777777777777</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -6036,7 +6033,7 @@
         <v>3</v>
       </c>
       <c r="B51">
-        <v>0.9554140127388535</v>
+        <v>0.91875</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -6044,7 +6041,7 @@
         <v>4</v>
       </c>
       <c r="B52">
-        <v>0.9903846153846154</v>
+        <v>0.9809523809523809</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -6052,7 +6049,7 @@
         <v>5</v>
       </c>
       <c r="B53">
-        <v>0.941747572815534</v>
+        <v>0.9603960396039604</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -6060,12 +6057,12 @@
         <v>6</v>
       </c>
       <c r="B54">
-        <v>1</v>
+        <v>0.9850746268656716</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -6081,15 +6078,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -6144,7 +6141,7 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9948955916473318</v>
+        <v>0.9944315545243619</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -6159,7 +6156,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.3806276049999724</v>
+        <v>0.4154801280000129</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -6168,23 +6165,23 @@
         <v>0.01</v>
       </c>
       <c r="M5">
-        <v>0.9925132328872037</v>
+        <v>0.9932433269064765</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6192,7 +6189,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9978118161925602</v>
+        <v>0.9989059080962801</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -6203,7 +6200,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9911894273127754</v>
+        <v>0.986784140969163</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -6214,7 +6211,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.994413407821229</v>
+        <v>0.9916201117318436</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -6225,7 +6222,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9935897435897436</v>
+        <v>1</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -6247,7 +6244,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>0.9900990099009901</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -6258,7 +6255,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>0.9705882352941176</v>
+        <v>0.9852941176470589</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -6266,18 +6263,18 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -6304,7 +6301,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6359,31 +6356,31 @@
         <v>0.95</v>
       </c>
       <c r="D4">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="E4">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>0.9535962877030162</v>
+        <v>0.951276102088167</v>
       </c>
       <c r="H4">
-        <v>0.04640371229698376</v>
+        <v>0.04872389791183294</v>
       </c>
       <c r="I4" t="s">
         <v>13</v>
       </c>
       <c r="J4">
-        <v>0.9610824551190823</v>
+        <v>0.9577474497896405</v>
       </c>
       <c r="L4">
         <v>4</v>
       </c>
       <c r="M4">
-        <v>0.9610824551190823</v>
+        <v>0.9577474497896404</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6435,41 +6432,41 @@
         <v>0.95</v>
       </c>
       <c r="D6">
-        <v>0.9633410672853828</v>
+        <v>0.9577726218097448</v>
       </c>
       <c r="E6">
-        <v>0.9633410672853828</v>
+        <v>0.9582366589327146</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0.9633410672853828</v>
+        <v>0.9582366589327146</v>
       </c>
       <c r="H6">
-        <v>0.03665893271461717</v>
+        <v>0.04176334106728538</v>
       </c>
       <c r="I6" t="s">
         <v>15</v>
       </c>
       <c r="J6">
-        <v>0.9641101485684878</v>
+        <v>0.9635694308832284</v>
       </c>
       <c r="L6">
         <v>4</v>
       </c>
       <c r="M6">
-        <v>0.9641101485684878</v>
+        <v>0.9635694308832286</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -6485,7 +6482,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6540,7 +6537,7 @@
         <v>0.95</v>
       </c>
       <c r="D4">
-        <v>0.9948955916473318</v>
+        <v>0.9944315545243619</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -6558,13 +6555,13 @@
         <v>13</v>
       </c>
       <c r="J4">
-        <v>0.9925132328872036</v>
+        <v>0.9932433269064765</v>
       </c>
       <c r="K4">
         <v>0.01</v>
       </c>
       <c r="M4">
-        <v>0.9925132328872037</v>
+        <v>0.9932433269064765</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6616,7 +6613,7 @@
         <v>0.95</v>
       </c>
       <c r="D6">
-        <v>0.9962877030162413</v>
+        <v>0.9944315545243619</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -6634,23 +6631,23 @@
         <v>15</v>
       </c>
       <c r="J6">
-        <v>0.9963725361616106</v>
+        <v>0.9928109972774349</v>
       </c>
       <c r="K6">
         <v>0.01</v>
       </c>
       <c r="M6">
-        <v>0.9963725361616106</v>
+        <v>0.9928109972774349</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -6717,7 +6714,7 @@
         <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -6813,7 +6810,7 @@
         <v>38</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -6828,15 +6825,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -6906,7 +6903,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1.501472937000017</v>
+        <v>1.644036248999953</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -6917,18 +6914,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -7010,18 +7007,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -7029,7 +7026,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
         <v>11530</v>
@@ -7040,7 +7037,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -7051,7 +7048,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -7062,7 +7059,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
         <v>17</v>
@@ -7073,13 +7070,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>1325</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -7087,7 +7084,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
         <v>2373</v>
@@ -7098,7 +7095,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
         <v>305</v>
@@ -7109,7 +7106,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
         <v>85760</v>
@@ -7117,27 +7114,27 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33">
-        <v>0.8901190088421045</v>
+        <v>0.890119070780596</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -7153,15 +7150,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -7231,7 +7228,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1.487060923999707</v>
+        <v>1.781241131999991</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -7242,18 +7239,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -7335,18 +7332,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -7354,7 +7351,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
         <v>13077</v>
@@ -7365,7 +7362,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -7376,7 +7373,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -7387,7 +7384,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
         <v>26</v>
@@ -7398,13 +7395,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>1300</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -7412,7 +7409,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
         <v>1816</v>
@@ -7423,7 +7420,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -7434,7 +7431,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
         <v>85091</v>
@@ -7442,15 +7439,15 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -7458,7 +7455,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.7918938085801932</v>
+        <v>0.7918937346333073</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -7466,7 +7463,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.8577086087094978</v>
+        <v>0.8577085616206699</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -7474,7 +7471,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.9384425667333275</v>
+        <v>0.9384426098877602</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -7482,7 +7479,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.962753093903993</v>
+        <v>0.9627530892941363</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -7490,7 +7487,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.9727721233566465</v>
+        <v>0.9727721283867071</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -7498,7 +7495,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.9603513662912506</v>
+        <v>0.9603513590991497</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -7506,17 +7503,17 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.8660019275733236</v>
+        <v>0.8660019464679389</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -7532,15 +7529,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -7610,7 +7607,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1.50854602399977</v>
+        <v>1.561271374</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -7621,18 +7618,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -7714,18 +7711,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -7733,10 +7730,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>12789</v>
+        <v>12788</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -7744,7 +7741,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -7755,7 +7752,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -7766,7 +7763,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
         <v>18</v>
@@ -7777,13 +7774,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>1199</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -7791,7 +7788,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
         <v>1783</v>
@@ -7802,7 +7799,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -7813,26 +7810,26 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>85521</v>
+        <v>85522</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7840,7 +7837,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.8128773458508067</v>
+        <v>0.8128771706103896</v>
       </c>
       <c r="C33">
         <v>3</v>
@@ -7851,7 +7848,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.8602594706556095</v>
+        <v>0.8602595533276644</v>
       </c>
       <c r="C34">
         <v>3</v>
@@ -7862,7 +7859,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.9512122126586209</v>
+        <v>0.9512122625305806</v>
       </c>
       <c r="C35">
         <v>4</v>
@@ -7873,7 +7870,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.9636066444865592</v>
+        <v>0.9636066382900544</v>
       </c>
       <c r="C36">
         <v>5</v>
@@ -7884,7 +7881,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.9755999726228438</v>
+        <v>0.9755999599585318</v>
       </c>
       <c r="C37">
         <v>5</v>
@@ -7895,7 +7892,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.9675369817256161</v>
+        <v>0.967536974305269</v>
       </c>
       <c r="C38">
         <v>4</v>
@@ -7906,7 +7903,7 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.8660019275733236</v>
+        <v>0.8660019464679389</v>
       </c>
       <c r="C39">
         <v>4</v>
@@ -7914,12 +7911,12 @@
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -7935,15 +7932,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8013,7 +8010,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>2.090471408999747</v>
+        <v>2.146093229999963</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -8027,18 +8024,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8120,15 +8117,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -8171,7 +8168,7 @@
         <v>2</v>
       </c>
       <c r="J25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -8192,15 +8189,15 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -8208,7 +8205,7 @@
         <v>0</v>
       </c>
       <c r="B32">
-        <v>0.9438114162172209</v>
+        <v>0.9438114007404317</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -8216,7 +8213,7 @@
         <v>1</v>
       </c>
       <c r="B33">
-        <v>0.8660019275733236</v>
+        <v>0.8660019464679389</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -8224,7 +8221,7 @@
         <v>2</v>
       </c>
       <c r="B34">
-        <v>0.8500615293419558</v>
+        <v>0.8500614022135595</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -8232,20 +8229,20 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>0.9603513662912506</v>
+        <v>0.9603513590991497</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -8282,15 +8279,15 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -8309,7 +8306,7 @@
         <v>0.5481132075471699</v>
       </c>
       <c r="J49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -8354,7 +8351,7 @@
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -8370,15 +8367,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8448,7 +8445,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.3882359640001596</v>
+        <v>0.390346610999984</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -8462,18 +8459,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8555,23 +8552,23 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21">
-        <v>0.8343723779709749</v>
+        <v>0.8343723718990144</v>
       </c>
       <c r="B21">
         <v>0.01</v>
@@ -8593,15 +8590,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8656,44 +8653,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9568445475638051</v>
+        <v>0.9651972157772621</v>
       </c>
       <c r="E5">
-        <v>0.9568445475638051</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9568445475638051</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="H5">
-        <v>0.0431554524361949</v>
+        <v>0.03387470997679815</v>
       </c>
       <c r="I5">
-        <v>1.526485220000268</v>
+        <v>1.610437100000013</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9546740538134185</v>
+        <v>0.9602859023151588</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8701,7 +8698,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9978118161925602</v>
+        <v>0.9956236323851203</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -8712,7 +8709,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9074889867841409</v>
+        <v>0.920704845814978</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -8723,7 +8720,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9022346368715084</v>
+        <v>0.9497206703910615</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -8734,7 +8731,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9487179487179487</v>
+        <v>0.9294871794871795</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -8775,18 +8772,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -8794,10 +8791,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>37900</v>
+        <v>37814</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -8805,10 +8802,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>13172</v>
+        <v>12745</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -8816,10 +8813,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>11160</v>
+        <v>12544</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -8827,10 +8824,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>3812</v>
+        <v>3674</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -8838,13 +8835,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>3146</v>
+        <v>3032</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -8852,10 +8849,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>3348</v>
+        <v>3640</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -8863,10 +8860,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>1801</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -8874,35 +8871,35 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>26971</v>
+        <v>25883</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33">
-        <v>0.03949081170352875</v>
+        <v>0.03911013995969781</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -8918,15 +8915,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8981,44 +8978,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9651972157772621</v>
+        <v>0.9573085846867749</v>
       </c>
       <c r="E5">
-        <v>0.965661252900232</v>
+        <v>0.9577726218097448</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.965661252900232</v>
+        <v>0.9577726218097448</v>
       </c>
       <c r="H5">
-        <v>0.03433874709976798</v>
+        <v>0.04222737819025522</v>
       </c>
       <c r="I5">
-        <v>1.469506139000259</v>
+        <v>1.589364872999965</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9656427257933603</v>
+        <v>0.9632547675729706</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -9026,7 +9023,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9617067833698031</v>
+        <v>0.9463894967177243</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -9048,7 +9045,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9776536312849162</v>
+        <v>0.9692737430167597</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -9059,7 +9056,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9487179487179487</v>
+        <v>0.9358974358974359</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -9081,7 +9078,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9603960396039604</v>
+        <v>0.9801980198019802</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -9100,18 +9097,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -9119,10 +9116,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>34185</v>
+        <v>34235</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -9130,10 +9127,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>13785</v>
+        <v>13772</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -9141,10 +9138,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>15107</v>
+        <v>13688</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -9152,10 +9149,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>3924</v>
+        <v>3949</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -9163,13 +9160,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>3193</v>
+        <v>3107</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -9177,10 +9174,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>3121</v>
+        <v>4357</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -9188,10 +9185,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>2055</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -9199,23 +9196,23 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>25940</v>
+        <v>26056</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -9223,7 +9220,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.0368939906793001</v>
+        <v>0.03703546924162571</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -9231,7 +9228,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.04020186647274582</v>
+        <v>0.04067535778323284</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -9239,7 +9236,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.06229990109438011</v>
+        <v>0.04158043355268359</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -9247,7 +9244,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.04123048188196521</v>
+        <v>0.04405834872490533</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -9255,7 +9252,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.04109783654352295</v>
+        <v>0.04137370179522182</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -9263,7 +9260,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.03674598561303999</v>
+        <v>0.05435002715128745</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -9271,17 +9268,17 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.06081736012957795</v>
+        <v>0.0557932543723958</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>